<commit_message>
Add Hyderabad to the travel map
Adds Hyderabad as a visited place, which brings in Telangana as a new
filled state (22 states/UTs now) with its own region page. Recorded in
Travels.xlsx as well, in both the place list and the region summary
column.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPzWfJYW89cbPigJgnC46N
</commit_message>
<xml_diff>
--- a/Travels.xlsx
+++ b/Travels.xlsx
@@ -374,7 +374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="42" customWidth="1" style="5" min="1" max="1"/>
@@ -1306,6 +1306,11 @@
           <t>Bihar</t>
         </is>
       </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="5">
       <c r="A53" s="2" t="inlineStr">
@@ -2963,7 +2968,18 @@
         </is>
       </c>
     </row>
-    <row r="191" ht="15.75" customHeight="1" s="5"/>
+    <row r="191" ht="15.75" customHeight="1" s="5">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+    </row>
     <row r="192" ht="15.75" customHeight="1" s="5"/>
     <row r="193" ht="15.75" customHeight="1" s="5"/>
     <row r="194" ht="15.75" customHeight="1" s="5"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ abhineet-agarwal/abhineet-agarwal.github.io@af95503db05565c7794cd8e7ab99f270c78c0668 🚀
</commit_message>
<xml_diff>
--- a/Travels.xlsx
+++ b/Travels.xlsx
@@ -374,7 +374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="42" customWidth="1" style="5" min="1" max="1"/>
@@ -1306,6 +1306,11 @@
           <t>Bihar</t>
         </is>
       </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="5">
       <c r="A53" s="2" t="inlineStr">
@@ -2963,7 +2968,18 @@
         </is>
       </c>
     </row>
-    <row r="191" ht="15.75" customHeight="1" s="5"/>
+    <row r="191" ht="15.75" customHeight="1" s="5">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+    </row>
     <row r="192" ht="15.75" customHeight="1" s="5"/>
     <row r="193" ht="15.75" customHeight="1" s="5"/>
     <row r="194" ht="15.75" customHeight="1" s="5"/>

</xml_diff>